<commit_message>
chore(radar): auto audit update 2026-08-17
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1132,6 +1132,655 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>729.87</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-0.0016</v>
+      </c>
+      <c r="E13" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>RVol: 0.66x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>225.01</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.0007000000000000001</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>RVol: 0.76x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>305.59</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.0011</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>RVol: 0.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>480.35</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.0304</v>
+      </c>
+      <c r="E16" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>261.31</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-0.0051</v>
+      </c>
+      <c r="E17" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>568.97</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-0.0354</v>
+      </c>
+      <c r="E18" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>RVol: 1.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>344</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-0.005500000000000001</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5.32</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>RVol: 0.58x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>339.3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.008699999999999999</v>
+      </c>
+      <c r="E20" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>RVol: 0.64x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1011.75</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.0413</v>
+      </c>
+      <c r="E21" t="n">
+        <v>40.87</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>536.01</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.0535</v>
+      </c>
+      <c r="E22" t="n">
+        <v>29.53</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>994.79</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.0219</v>
+      </c>
+      <c r="E23" t="n">
+        <v>35.36</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-18
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1781,6 +1781,655 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>717.51</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-0.0169</v>
+      </c>
+      <c r="E24" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>RVol: 1.23x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>219.74</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-0.0234</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>310.03</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.0145</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>RVol: 1.00x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>481.63</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="E27" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>RVol: 0.63x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>259.45</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.0071</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>RVol: 0.68x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>543.67</v>
+      </c>
+      <c r="D29" t="n">
+        <v>-0.0445</v>
+      </c>
+      <c r="E29" t="n">
+        <v>17.45</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>RVol: 1.66x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>344.2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>RVol: 0.62x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>336.87</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-0.0072</v>
+      </c>
+      <c r="E31" t="n">
+        <v>9.41</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>RVol: 0.71x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>940.76</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-0.0702</v>
+      </c>
+      <c r="E32" t="n">
+        <v>52.03</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>RVol: 0.88x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>496.16</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-0.07429999999999999</v>
+      </c>
+      <c r="E33" t="n">
+        <v>29.77</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>RVol: 1.10x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>903.6799999999999</v>
+      </c>
+      <c r="D34" t="n">
+        <v>-0.0916</v>
+      </c>
+      <c r="E34" t="n">
+        <v>62.59</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-19
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2430,6 +2430,655 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>716.08</v>
+      </c>
+      <c r="D35" t="n">
+        <v>-0.002</v>
+      </c>
+      <c r="E35" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>RVol: 0.87x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>217.56</v>
+      </c>
+      <c r="D36" t="n">
+        <v>-0.009899999999999999</v>
+      </c>
+      <c r="E36" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>316.83</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.0219</v>
+      </c>
+      <c r="E37" t="n">
+        <v>9.68</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>484.31</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.005600000000000001</v>
+      </c>
+      <c r="E38" t="n">
+        <v>9.94</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>RVol: 0.52x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>265.84</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.0246</v>
+      </c>
+      <c r="E39" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>546.03</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="E40" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>RVol: 0.98x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>344.72</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="E41" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>RVol: 0.64x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>351.12</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.0423</v>
+      </c>
+      <c r="E42" t="n">
+        <v>15.92</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>937.1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>-0.0039</v>
+      </c>
+      <c r="E43" t="n">
+        <v>44.82</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>RVol: 0.64x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>462.09</v>
+      </c>
+      <c r="D44" t="n">
+        <v>-0.0687</v>
+      </c>
+      <c r="E44" t="n">
+        <v>39.72</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>832.5599999999999</v>
+      </c>
+      <c r="D45" t="n">
+        <v>-0.07870000000000001</v>
+      </c>
+      <c r="E45" t="n">
+        <v>86.05</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>RVol: 1.07x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-20
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3079,6 +3079,655 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>710.9299999999999</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-0.0072</v>
+      </c>
+      <c r="E46" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>RVol: 0.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>216.85</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-0.0033</v>
+      </c>
+      <c r="E47" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>RVol: 0.76x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>311.3</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-0.0175</v>
+      </c>
+      <c r="E48" t="n">
+        <v>9.630000000000001</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>481.15</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-0.006500000000000001</v>
+      </c>
+      <c r="E49" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>RVol: 0.49x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>260.11</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-0.0216</v>
+      </c>
+      <c r="E50" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>RVol: 0.57x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>545.83</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-0.0004</v>
+      </c>
+      <c r="E51" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>340.67</v>
+      </c>
+      <c r="D52" t="n">
+        <v>-0.0117</v>
+      </c>
+      <c r="E52" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>RVol: 0.62x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>345.13</v>
+      </c>
+      <c r="D53" t="n">
+        <v>-0.0171</v>
+      </c>
+      <c r="E53" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>RVol: 0.76x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>974.33</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.0397</v>
+      </c>
+      <c r="E54" t="n">
+        <v>48.21</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>RVol: 0.61x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>469.05</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.0151</v>
+      </c>
+      <c r="E55" t="n">
+        <v>23.58</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>RVol: 0.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>850.24</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="E56" t="n">
+        <v>42.11</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>RVol: 0.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-21
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M56"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3728,6 +3728,655 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>713.4400000000001</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0.0035</v>
+      </c>
+      <c r="E57" t="n">
+        <v>6.47</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>RVol: 0.82x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>214.72</v>
+      </c>
+      <c r="D58" t="n">
+        <v>-0.0098</v>
+      </c>
+      <c r="E58" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>RVol: 0.84x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>309.35</v>
+      </c>
+      <c r="D59" t="n">
+        <v>-0.0063</v>
+      </c>
+      <c r="E59" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>483.24</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="E60" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>RVol: 0.58x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>258.63</v>
+      </c>
+      <c r="D61" t="n">
+        <v>-0.005699999999999999</v>
+      </c>
+      <c r="E61" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>549.9</v>
+      </c>
+      <c r="D62" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="E62" t="n">
+        <v>10.64</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>RVol: 0.76x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>344.82</v>
+      </c>
+      <c r="D63" t="n">
+        <v>0.0122</v>
+      </c>
+      <c r="E63" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>RVol: 0.76x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>362.86</v>
+      </c>
+      <c r="D64" t="n">
+        <v>0.05139999999999999</v>
+      </c>
+      <c r="E64" t="n">
+        <v>19.6</v>
+      </c>
+      <c r="F64" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>RVol: 1.66x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>966.78</v>
+      </c>
+      <c r="D65" t="n">
+        <v>-0.0077</v>
+      </c>
+      <c r="E65" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>RVol: 0.52x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>459.44</v>
+      </c>
+      <c r="D66" t="n">
+        <v>-0.0205</v>
+      </c>
+      <c r="E66" t="n">
+        <v>24.47</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>RVol: 0.51x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>850</v>
+      </c>
+      <c r="D67" t="n">
+        <v>-0.0003</v>
+      </c>
+      <c r="E67" t="n">
+        <v>35.49</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>RVol: 0.53x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-24
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4377,6 +4377,655 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>706.3200000000001</v>
+      </c>
+      <c r="D68" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="E68" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>RVol: 0.93x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>208.48</v>
+      </c>
+      <c r="D69" t="n">
+        <v>-0.0291</v>
+      </c>
+      <c r="E69" t="n">
+        <v>8.34</v>
+      </c>
+      <c r="F69" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>RVol: 1.13x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>310.34</v>
+      </c>
+      <c r="D70" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="E70" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>RVol: 0.61x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>487.31</v>
+      </c>
+      <c r="D71" t="n">
+        <v>0.008399999999999999</v>
+      </c>
+      <c r="E71" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>RVol: 0.43x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>262.07</v>
+      </c>
+      <c r="D72" t="n">
+        <v>0.0133</v>
+      </c>
+      <c r="E72" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>RVol: 0.58x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>559.02</v>
+      </c>
+      <c r="D73" t="n">
+        <v>0.0166</v>
+      </c>
+      <c r="E73" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>348.06</v>
+      </c>
+      <c r="D74" t="n">
+        <v>0.009399999999999999</v>
+      </c>
+      <c r="E74" t="n">
+        <v>9.109999999999999</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>RVol: 0.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>348.95</v>
+      </c>
+      <c r="D75" t="n">
+        <v>-0.0383</v>
+      </c>
+      <c r="E75" t="n">
+        <v>14.98</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>RVol: 1.11x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>910.4299999999999</v>
+      </c>
+      <c r="D76" t="n">
+        <v>-0.0583</v>
+      </c>
+      <c r="E76" t="n">
+        <v>48.85</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>435.38</v>
+      </c>
+      <c r="D77" t="n">
+        <v>-0.0524</v>
+      </c>
+      <c r="E77" t="n">
+        <v>27.45</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>RVol: 0.91x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>794.65</v>
+      </c>
+      <c r="D78" t="n">
+        <v>-0.06509999999999999</v>
+      </c>
+      <c r="E78" t="n">
+        <v>48.74</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>RVol: 0.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-25
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M78"/>
+  <dimension ref="A1:M89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5026,6 +5026,655 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>710.72</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="E79" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>RVol: 0.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>213.05</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0.0219</v>
+      </c>
+      <c r="E80" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="F80" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>RVol: 1.03x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>309.9</v>
+      </c>
+      <c r="D81" t="n">
+        <v>-0.0014</v>
+      </c>
+      <c r="E81" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>RVol: 0.49x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>491.71</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="E82" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>RVol: 0.52x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>261.06</v>
+      </c>
+      <c r="D83" t="n">
+        <v>-0.0039</v>
+      </c>
+      <c r="E83" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>RVol: 0.53x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>570.05</v>
+      </c>
+      <c r="D84" t="n">
+        <v>0.0197</v>
+      </c>
+      <c r="E84" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>RVol: 0.55x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>346.96</v>
+      </c>
+      <c r="D85" t="n">
+        <v>-0.0032</v>
+      </c>
+      <c r="E85" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>350.25</v>
+      </c>
+      <c r="D86" t="n">
+        <v>0.0037</v>
+      </c>
+      <c r="E86" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>932.97</v>
+      </c>
+      <c r="D87" t="n">
+        <v>0.0248</v>
+      </c>
+      <c r="E87" t="n">
+        <v>30.37</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>RVol: 0.49x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>450.75</v>
+      </c>
+      <c r="D88" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="E88" t="n">
+        <v>21.66</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>RVol: 0.53x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>821.67</v>
+      </c>
+      <c r="D89" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="E89" t="n">
+        <v>25.88</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>RVol: 0.49x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-27
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M89"/>
+  <dimension ref="A1:M100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5675,6 +5675,655 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>711.37</v>
+      </c>
+      <c r="D90" t="n">
+        <v>0.0009</v>
+      </c>
+      <c r="E90" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>RVol: 0.54x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>209.66</v>
+      </c>
+      <c r="D91" t="n">
+        <v>-0.0159</v>
+      </c>
+      <c r="E91" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="F91" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>RVol: 1.56x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>313.45</v>
+      </c>
+      <c r="D92" t="n">
+        <v>0.0115</v>
+      </c>
+      <c r="E92" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>RVol: 0.67x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>496.37</v>
+      </c>
+      <c r="D93" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="E93" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>RVol: 0.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>260.28</v>
+      </c>
+      <c r="D94" t="n">
+        <v>-0.003</v>
+      </c>
+      <c r="E94" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>RVol: 0.46x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>576.14</v>
+      </c>
+      <c r="D95" t="n">
+        <v>0.0107</v>
+      </c>
+      <c r="E95" t="n">
+        <v>31.46</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Lower Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>STOPPING VOLUME 🛑</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Long Trigger 🚀</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>RVol: 1.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>342</v>
+      </c>
+      <c r="D96" t="n">
+        <v>-0.0143</v>
+      </c>
+      <c r="E96" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>RVol: 0.78x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>345.82</v>
+      </c>
+      <c r="D97" t="n">
+        <v>-0.0126</v>
+      </c>
+      <c r="E97" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>938.4</v>
+      </c>
+      <c r="D98" t="n">
+        <v>0.0058</v>
+      </c>
+      <c r="E98" t="n">
+        <v>21.15</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>RVol: 0.52x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>468.88</v>
+      </c>
+      <c r="D99" t="n">
+        <v>0.04019999999999999</v>
+      </c>
+      <c r="E99" t="n">
+        <v>21.99</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>RVol: 0.62x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>846.37</v>
+      </c>
+      <c r="D100" t="n">
+        <v>0.0301</v>
+      </c>
+      <c r="E100" t="n">
+        <v>30.02</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>RVol: 0.44x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-28
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M100"/>
+  <dimension ref="A1:M111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6324,6 +6324,655 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>721.11</v>
+      </c>
+      <c r="D101" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="E101" t="n">
+        <v>6.83</v>
+      </c>
+      <c r="F101" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>227.98</v>
+      </c>
+      <c r="D102" t="n">
+        <v>0.08740000000000001</v>
+      </c>
+      <c r="E102" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F102" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>RVol: 2.56x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>314.58</v>
+      </c>
+      <c r="D103" t="n">
+        <v>0.0036</v>
+      </c>
+      <c r="E103" t="n">
+        <v>6</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>RVol: 0.65x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>505.06</v>
+      </c>
+      <c r="D104" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="E104" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>RVol: 0.84x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>256.26</v>
+      </c>
+      <c r="D105" t="n">
+        <v>-0.0154</v>
+      </c>
+      <c r="E105" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>571.1</v>
+      </c>
+      <c r="D106" t="n">
+        <v>-0.008699999999999999</v>
+      </c>
+      <c r="E106" t="n">
+        <v>20.77</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>RVol: 0.86x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>340.65</v>
+      </c>
+      <c r="D107" t="n">
+        <v>-0.0039</v>
+      </c>
+      <c r="E107" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>RVol: 0.91x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>354.81</v>
+      </c>
+      <c r="D108" t="n">
+        <v>0.026</v>
+      </c>
+      <c r="E108" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>935.39</v>
+      </c>
+      <c r="D109" t="n">
+        <v>-0.0032</v>
+      </c>
+      <c r="E109" t="n">
+        <v>61.82</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>RVol: 0.86x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>462</v>
+      </c>
+      <c r="D110" t="n">
+        <v>-0.0147</v>
+      </c>
+      <c r="E110" t="n">
+        <v>36.83</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>847.2</v>
+      </c>
+      <c r="D111" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="E111" t="n">
+        <v>62.81</v>
+      </c>
+      <c r="F111" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>RVol: 1.08x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-08-29
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M111"/>
+  <dimension ref="A1:M122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6973,6 +6973,655 @@
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>716.4299999999999</v>
+      </c>
+      <c r="D112" t="n">
+        <v>-0.006500000000000001</v>
+      </c>
+      <c r="E112" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="F112" t="n">
+        <v>1</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>RVol: 1.00x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>217.55</v>
+      </c>
+      <c r="D113" t="n">
+        <v>-0.0457</v>
+      </c>
+      <c r="E113" t="n">
+        <v>12.45</v>
+      </c>
+      <c r="F113" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>RVol: 1.56x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>319.7</v>
+      </c>
+      <c r="D114" t="n">
+        <v>0.0163</v>
+      </c>
+      <c r="E114" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>RVol: 0.81x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>513.53</v>
+      </c>
+      <c r="D115" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="E115" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>266.43</v>
+      </c>
+      <c r="D116" t="n">
+        <v>0.0397</v>
+      </c>
+      <c r="E116" t="n">
+        <v>9.779999999999999</v>
+      </c>
+      <c r="F116" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>RVol: 1.17x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>578.02</v>
+      </c>
+      <c r="D117" t="n">
+        <v>0.0121</v>
+      </c>
+      <c r="E117" t="n">
+        <v>18.19</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>RVol: 0.98x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>346.59</v>
+      </c>
+      <c r="D118" t="n">
+        <v>0.0174</v>
+      </c>
+      <c r="E118" t="n">
+        <v>8.869999999999999</v>
+      </c>
+      <c r="F118" t="n">
+        <v>1</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>RVol: 1.00x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>348.75</v>
+      </c>
+      <c r="D119" t="n">
+        <v>-0.0171</v>
+      </c>
+      <c r="E119" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>RVol: 0.99x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>932.86</v>
+      </c>
+      <c r="D120" t="n">
+        <v>-0.0027</v>
+      </c>
+      <c r="E120" t="n">
+        <v>37.71</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>RVol: 0.72x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>459.45</v>
+      </c>
+      <c r="D121" t="n">
+        <v>-0.005500000000000001</v>
+      </c>
+      <c r="E121" t="n">
+        <v>19.94</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>RVol: 0.53x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>829.76</v>
+      </c>
+      <c r="D122" t="n">
+        <v>-0.0206</v>
+      </c>
+      <c r="E122" t="n">
+        <v>30.08</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>RVol: 0.64x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-01
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M122"/>
+  <dimension ref="A1:M133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7622,6 +7622,655 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>716.76</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="E123" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>220.78</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0.0148</v>
+      </c>
+      <c r="E124" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>RVol: 0.95x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>316.85</v>
+      </c>
+      <c r="D125" t="n">
+        <v>-0.0089</v>
+      </c>
+      <c r="E125" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>507.29</v>
+      </c>
+      <c r="D126" t="n">
+        <v>-0.0122</v>
+      </c>
+      <c r="E126" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>RVol: 0.90x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>259.77</v>
+      </c>
+      <c r="D127" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="E127" t="n">
+        <v>7.24</v>
+      </c>
+      <c r="F127" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>RVol: 1.18x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>572.34</v>
+      </c>
+      <c r="D128" t="n">
+        <v>-0.0098</v>
+      </c>
+      <c r="E128" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>RVol: 0.80x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>339.35</v>
+      </c>
+      <c r="D129" t="n">
+        <v>-0.0209</v>
+      </c>
+      <c r="E129" t="n">
+        <v>7.43</v>
+      </c>
+      <c r="F129" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>RVol: 1.30x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>367.95</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0.0551</v>
+      </c>
+      <c r="E130" t="n">
+        <v>21.77</v>
+      </c>
+      <c r="F130" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>RVol: 1.84x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>958.73</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0.0277</v>
+      </c>
+      <c r="E131" t="n">
+        <v>29.18</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>450.55</v>
+      </c>
+      <c r="D132" t="n">
+        <v>-0.0194</v>
+      </c>
+      <c r="E132" t="n">
+        <v>14.93</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>828.38</v>
+      </c>
+      <c r="D133" t="n">
+        <v>-0.0017</v>
+      </c>
+      <c r="E133" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="F133" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>RVol: 0.77x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-02
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M144"/>
+  <dimension ref="A1:M155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8920,6 +8920,655 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>709.24</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="E145" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>224.41</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0.0321</v>
+      </c>
+      <c r="E146" t="n">
+        <v>9.470000000000001</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>RVol: 1.21x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>324.96</v>
+      </c>
+      <c r="D147" t="n">
+        <v>-0.0005</v>
+      </c>
+      <c r="E147" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>RVol: 0.83x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>496.82</v>
+      </c>
+      <c r="D148" t="n">
+        <v>-0.008399999999999999</v>
+      </c>
+      <c r="E148" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="F148" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>RVol: 0.59x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>254.98</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="E149" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="F149" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>NR7 (7日极窄)</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>RVol: 0.69x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>592.85</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0.0247</v>
+      </c>
+      <c r="E150" t="n">
+        <v>23.38</v>
+      </c>
+      <c r="F150" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>RVol: 1.02x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>337.12</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="E151" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>RVol: 0.89x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>357.01</v>
+      </c>
+      <c r="D152" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="E152" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>956.08</v>
+      </c>
+      <c r="D153" t="n">
+        <v>0.0243</v>
+      </c>
+      <c r="E153" t="n">
+        <v>30.84</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>RVol: 0.73x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>448.9</v>
+      </c>
+      <c r="D154" t="n">
+        <v>-0.0034</v>
+      </c>
+      <c r="E154" t="n">
+        <v>19.58</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>RVol: 0.52x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>808.54</v>
+      </c>
+      <c r="D155" t="n">
+        <v>-0.009899999999999999</v>
+      </c>
+      <c r="E155" t="n">
+        <v>49.74</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>RVol: 0.66x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-03
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M155"/>
+  <dimension ref="A1:M166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9569,6 +9569,655 @@
         </is>
       </c>
     </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>717.67</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0.0119</v>
+      </c>
+      <c r="E156" t="n">
+        <v>9.220000000000001</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>228.45</v>
+      </c>
+      <c r="D157" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="E157" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="F157" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>RVol: 1.04x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>328.21</v>
+      </c>
+      <c r="D158" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E158" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F158" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>RVol: 0.92x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>510.12</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0.0268</v>
+      </c>
+      <c r="E159" t="n">
+        <v>14.85</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>RVol: 0.98x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>258.9</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0.0154</v>
+      </c>
+      <c r="E160" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>RVol: 0.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>610.6799999999999</v>
+      </c>
+      <c r="D161" t="n">
+        <v>0.0301</v>
+      </c>
+      <c r="E161" t="n">
+        <v>15.11</v>
+      </c>
+      <c r="F161" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>RVol: 1.23x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>342.48</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0.0159</v>
+      </c>
+      <c r="E162" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="F162" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>376.36</v>
+      </c>
+      <c r="D163" t="n">
+        <v>0.0542</v>
+      </c>
+      <c r="E163" t="n">
+        <v>18.22</v>
+      </c>
+      <c r="F163" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Upper Wick Rejection</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>TOPPING OUT 🛑</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>VETO 🛑</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Sit on Hands (一票否决) 🔒</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>RVol: 1.79x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>958.16</v>
+      </c>
+      <c r="D164" t="n">
+        <v>0.0022</v>
+      </c>
+      <c r="E164" t="n">
+        <v>40.88</v>
+      </c>
+      <c r="F164" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>441.57</v>
+      </c>
+      <c r="D165" t="n">
+        <v>-0.0163</v>
+      </c>
+      <c r="E165" t="n">
+        <v>28.59</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>798.61</v>
+      </c>
+      <c r="D166" t="n">
+        <v>-0.0123</v>
+      </c>
+      <c r="E166" t="n">
+        <v>43.55</v>
+      </c>
+      <c r="F166" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>RVol: 0.75x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(radar): auto audit update 2026-09-04
</commit_message>
<xml_diff>
--- a/NQ_RADAR_Daily_Tracker.xlsx
+++ b/NQ_RADAR_Daily_Tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M166"/>
+  <dimension ref="A1:M177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10218,6 +10218,655 @@
         </is>
       </c>
     </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>718.96</v>
+      </c>
+      <c r="D167" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="E167" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="F167" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>RVol: 1.05x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>230.36</v>
+      </c>
+      <c r="D168" t="n">
+        <v>0.008399999999999999</v>
+      </c>
+      <c r="E168" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="F168" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>RVol: 1.04x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>319.97</v>
+      </c>
+      <c r="D169" t="n">
+        <v>-0.0251</v>
+      </c>
+      <c r="E169" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="F169" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>RVol: 0.97x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>499.7</v>
+      </c>
+      <c r="D170" t="n">
+        <v>-0.0204</v>
+      </c>
+      <c r="E170" t="n">
+        <v>11.64</v>
+      </c>
+      <c r="F170" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>RVol: 0.74x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>258.51</v>
+      </c>
+      <c r="D171" t="n">
+        <v>-0.0015</v>
+      </c>
+      <c r="E171" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="F171" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>RVol: 0.91x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>616.77</v>
+      </c>
+      <c r="D172" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E172" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="F172" t="n">
+        <v>1</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>Inside Bar (孕线)</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>Tight Compression ⚡</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>RVol: 1.00x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>338.46</v>
+      </c>
+      <c r="D173" t="n">
+        <v>-0.0117</v>
+      </c>
+      <c r="E173" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="F173" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>RVol: 0.94x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>354.08</v>
+      </c>
+      <c r="D174" t="n">
+        <v>-0.0592</v>
+      </c>
+      <c r="E174" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="F174" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>RVol: 1.76x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>1016.59</v>
+      </c>
+      <c r="D175" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="E175" t="n">
+        <v>48.77</v>
+      </c>
+      <c r="F175" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>RVol: 1.26x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>467.46</v>
+      </c>
+      <c r="D176" t="n">
+        <v>0.05860000000000001</v>
+      </c>
+      <c r="E176" t="n">
+        <v>26.04</v>
+      </c>
+      <c r="F176" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>RVol: 0.85x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>849.28</v>
+      </c>
+      <c r="D177" t="n">
+        <v>0.0634</v>
+      </c>
+      <c r="E177" t="n">
+        <v>47.97</v>
+      </c>
+      <c r="F177" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Normal Body</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Normal Volume</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>PASS ✅</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Watch &amp; Wait 🔒</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>RVol: 0.67x | 自动定时审计</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>